<commit_message>
additional search for 2025 and 2026
</commit_message>
<xml_diff>
--- a/data/screening/searchstrings and results.xlsx
+++ b/data/screening/searchstrings and results.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j_stee03\Sciebo\Review take off\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j_stee03\Uni\takeoff\data\screening\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C2344F3-1309-4821-999D-CA73AE53E8D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{051A5D55-81C9-418A-8B56-ECD78EC6EC68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-3585" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -29,12 +29,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="31">
   <si>
     <t>string</t>
   </si>
@@ -121,6 +124,12 @@
   </si>
   <si>
     <t>(Drone OR UAV OR UAS OR unmanned)  AND (biomass  OR shrub OR bush OR nitrogen OR ruderal OR disturbance OR reforestation OR grass OR drainage OR water OR moisture OR biodiversity OR canopy OR herb OR heterogeneity  OR ndvi OR nitrogen OR soil OR degradation OR diversity OR species OR vegetation OR cover) AND (grassland OR heather OR bog OR fen OR steppe OR floodplain OR meadow OR pasture OR peatland OR heathland)</t>
+  </si>
+  <si>
+    <t>new search on 03.03.2026 to search for articles since 25.04.2025</t>
+  </si>
+  <si>
+    <t>1092 results after deduplication in litseachr, 177 additional articles from 2025 and 2026 were identified</t>
   </si>
 </sst>
 </file>
@@ -455,21 +464,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="43.33203125" customWidth="1"/>
-    <col min="2" max="2" width="14.77734375" customWidth="1"/>
-    <col min="3" max="3" width="10.5546875" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5546875" customWidth="1"/>
-    <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.88671875" customWidth="1"/>
-    <col min="8" max="8" width="21.77734375" customWidth="1"/>
-    <col min="9" max="9" width="13.109375" customWidth="1"/>
+    <col min="1" max="1" width="43.28515625" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" customWidth="1"/>
+    <col min="8" max="8" width="21.7109375" customWidth="1"/>
+    <col min="9" max="9" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -498,7 +507,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="98.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="98.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -524,7 +533,7 @@
         <v>45769</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="145.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="145.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>14</v>
       </c>
@@ -550,7 +559,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="172.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="172.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>16</v>
       </c>
@@ -579,7 +588,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="152.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="152.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>17</v>
       </c>
@@ -608,7 +617,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="160.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="160.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -637,7 +646,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="150" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>19</v>
       </c>
@@ -666,7 +675,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="144" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="165" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>28</v>
       </c>
@@ -693,6 +702,26 @@
       </c>
       <c r="I8" s="1" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9">
+        <v>1039</v>
+      </c>
+      <c r="E9">
+        <v>754</v>
+      </c>
+      <c r="G9">
+        <v>1092</v>
+      </c>
+      <c r="H9" s="2">
+        <v>46084</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>